<commit_message>
Modifed domain entities to remove IEPAssociation from the key and instead move to a required resource
</commit_message>
<xml_diff>
--- a/MetaEdOutput/Documentation/Ed-Fi-Handbook/Ed-Fi-Handbook.xlsx
+++ b/MetaEdOutput/Documentation/Ed-Fi-Handbook/Ed-Fi-Handbook.xlsx
@@ -18494,11 +18494,11 @@
 Student (identity)
 StudentIEPAssociationID (identity)
 Used By:
-IEPGoal.StudentIEPAssociation (as identity)
-IEPServiceDelivery.StudentIEPAssociation (as identity)
-IEPServicePrescription.StudentIEPAssociation (as identity)
-StudentIEPAccommodation.StudentIEPAssociation (as identity)
-StudentIEPDisability.StudentIEPAssociation (as identity)</t>
+IEPGoal.StudentIEPAssociation (as required)
+IEPServiceDelivery.StudentIEPAssociation (as required)
+IEPServicePrescription.StudentIEPAssociation (as required)
+StudentIEPAccommodation.StudentIEPAssociation (as required)
+StudentIEPDisability.StudentIEPAssociation (as required)</t>
   </si>
   <si>
     <t xml:space="preserve">sedm.StudentIEPAssociation
@@ -19003,32 +19003,29 @@
 IEPGoalDetails (required)
 IEPGoalID (identity)
 Student (identity)
-StudentIEPAssociation (identity)
+StudentIEPAssociation (required)
 Used By:
 IEPGoal.IEPGoal (as required)</t>
   </si>
   <si>
     <t xml:space="preserve">sedm.IEPGoal
-IEPFinalizedDate [DATE] NOT NULL
-IEPGoalID [NVARCHAR](30) NOT NULL
-IEPServicingEducationOrganizationId [BIGINT] NOT NULL
-StudentIEPAssociationID [NVARCHAR](1024) NOT NULL
+IEPGoalID [NVARCHAR](256) NOT NULL
 StudentUSI [INT] NOT NULL
 EducationOrganizationId [BIGINT] NULL
 GoalAchievementPeriodBeginDate [DATE] NULL
 GoalAchievementPeriodEndDate [DATE] NULL
 IDEAEventDescriptorId [INT] NULL
 IDEAEventID [NVARCHAR](1024) NULL
+IEPFinalizedDate [DATE] NOT NULL
 IEPGoalDescriptorId [INT] NOT NULL
 IEPGoalDetails [NVARCHAR](2048) NOT NULL
+IEPServicingEducationOrganizationId [BIGINT] NOT NULL
+StudentIEPAssociationID [NVARCHAR](1024) NOT NULL
 CreateDate [DATETIME] NOT NULL
 LastModifiedDate [DATETIME] NOT NULL
 Id [UNIQUEIDENTIFIER] NOT NULL
 Primary Keys:
-IEPFinalizedDate
 IEPGoalID
-IEPServicingEducationOrganizationId
-StudentIEPAssociationID
 StudentUSI
 </t>
   </si>
@@ -19049,42 +19046,36 @@
 ServiceProvider (optional)
 Staff (optional)
 Student (identity)
-StudentIEPAssociation (identity)</t>
+StudentIEPAssociation (required)</t>
   </si>
   <si>
     <t xml:space="preserve">sedm.IEPServiceDelivery
-IEPFinalizedDate [DATE] NOT NULL
 IEPServiceDeliveryID [NVARCHAR](1024) NOT NULL
-IEPServicingEducationOrganizationId [BIGINT] NOT NULL
 ServiceDeliveryDate [DATE] NOT NULL
 ServiceDeliveryDescriptorId [INT] NOT NULL
-StudentIEPAssociationID [NVARCHAR](1024) NOT NULL
 StudentUSI [INT] NOT NULL
 EducationOrganizationId [BIGINT] NULL
 IDEAEventDescriptorId [INT] NULL
 IDEAEventID [NVARCHAR](1024) NULL
+IEPFinalizedDate [DATE] NOT NULL
+IEPServicingEducationOrganizationId [BIGINT] NOT NULL
 ServiceDeliveryStaffUSI [INT] NULL
 ServicePrescriptionDate [DATE] NULL
 ServicePrescriptionDescriptorId [INT] NULL
 ServiceProviderDescriptorId [INT] NULL
+StudentIEPAssociationID [NVARCHAR](1024) NOT NULL
 CreateDate [DATETIME] NOT NULL
 LastModifiedDate [DATETIME] NOT NULL
 Id [UNIQUEIDENTIFIER] NOT NULL
 Primary Keys:
-IEPFinalizedDate
 IEPServiceDeliveryID
-IEPServicingEducationOrganizationId
 ServiceDeliveryDate
 ServiceDeliveryDescriptorId
-StudentIEPAssociationID
 StudentUSI
 sedm.IEPServiceDeliveryExternalServiceProvider
-IEPFinalizedDate [DATE] NOT NULL
 IEPServiceDeliveryID [NVARCHAR](1024) NOT NULL
-IEPServicingEducationOrganizationId [BIGINT] NOT NULL
 ServiceDeliveryDate [DATE] NOT NULL
 ServiceDeliveryDescriptorId [INT] NOT NULL
-StudentIEPAssociationID [NVARCHAR](1024) NOT NULL
 StudentUSI [INT] NOT NULL
 ProviderCode [NVARCHAR](1024) NOT NULL
 ProviderFirstName [NVARCHAR](1024) NOT NULL
@@ -19093,12 +19084,9 @@
 ProviderMiddleName [NVARCHAR](1024) NULL
 CreateDate [DATETIME] NOT NULL
 Primary Keys:
-IEPFinalizedDate
 IEPServiceDeliveryID
-IEPServicingEducationOrganizationId
 ServiceDeliveryDate
 ServiceDeliveryDescriptorId
-StudentIEPAssociationID
 StudentUSI
 ProviderCode
 ProviderFirstName
@@ -19126,17 +19114,14 @@
 ServicePrescriptionDate (identity)
 Staff (optional)
 Student (identity)
-StudentIEPAssociation (identity)
+StudentIEPAssociation (required)
 Used By:
 IEPServiceDelivery.IEPServicePrescription (as optional)</t>
   </si>
   <si>
     <t xml:space="preserve">sedm.IEPServicePrescription
-IEPFinalizedDate [DATE] NOT NULL
-IEPServicingEducationOrganizationId [BIGINT] NOT NULL
 ServicePrescriptionDate [DATE] NOT NULL
 ServicePrescriptionDescriptorId [INT] NOT NULL
-StudentIEPAssociationID [NVARCHAR](1024) NOT NULL
 StudentUSI [INT] NOT NULL
 BeginDate [DATE] NOT NULL
 DurationMinutes [DECIMAL](5, 2) NOT NULL
@@ -19147,18 +19132,18 @@
 FrequencyValue [DECIMAL](5, 2) NOT NULL
 IDEAEventDescriptorId [INT] NULL
 IDEAEventID [NVARCHAR](1024) NULL
+IEPFinalizedDate [DATE] NOT NULL
+IEPServicingEducationOrganizationId [BIGINT] NOT NULL
 ServiceLocationTypeDescriptorId [INT] NOT NULL
 ServiceProvidingEducationOrganizationId [BIGINT] NULL
 StaffUSI [INT] NULL
+StudentIEPAssociationID [NVARCHAR](1024) NOT NULL
 CreateDate [DATETIME] NOT NULL
 LastModifiedDate [DATETIME] NOT NULL
 Id [UNIQUEIDENTIFIER] NOT NULL
 Primary Keys:
-IEPFinalizedDate
-IEPServicingEducationOrganizationId
 ServicePrescriptionDate
 ServicePrescriptionDescriptorId
-StudentIEPAssociationID
 StudentUSI
 </t>
   </si>
@@ -19173,34 +19158,28 @@
 Accommodation (required collection)
 EducationOrganization (identity)
 Student (identity)
-StudentIEPAssociation (identity)</t>
+StudentIEPAssociation (required)</t>
   </si>
   <si>
     <t xml:space="preserve">sedm.StudentIEPAccommodation
-IEPFinalizedDate [DATE] NOT NULL
 IEPServicingEducationOrganizationId [BIGINT] NOT NULL
-StudentIEPAssociationID [NVARCHAR](1024) NOT NULL
 StudentUSI [INT] NOT NULL
 AccommodationDescriptorId [INT] NOT NULL
 CreateDate [DATETIME] NOT NULL
 Primary Keys:
-IEPFinalizedDate
 IEPServicingEducationOrganizationId
-StudentIEPAssociationID
 StudentUSI
 AccommodationDescriptorId
 sedm.StudentIEPAccommodation
+IEPServicingEducationOrganizationId [BIGINT] NOT NULL
+StudentUSI [INT] NOT NULL
 IEPFinalizedDate [DATE] NOT NULL
-IEPServicingEducationOrganizationId [BIGINT] NOT NULL
 StudentIEPAssociationID [NVARCHAR](1024) NOT NULL
-StudentUSI [INT] NOT NULL
 CreateDate [DATETIME] NOT NULL
 LastModifiedDate [DATETIME] NOT NULL
 Id [UNIQUEIDENTIFIER] NOT NULL
 Primary Keys:
-IEPFinalizedDate
 IEPServicingEducationOrganizationId
-StudentIEPAssociationID
 StudentUSI
 </t>
   </si>
@@ -19215,26 +19194,11 @@
 Disability (required collection)
 EducationOrganization (identity)
 Student (identity)
-StudentIEPAssociation (identity)</t>
+StudentIEPAssociation (required)</t>
   </si>
   <si>
     <t xml:space="preserve">sedm.StudentIEPDisability
-IEPFinalizedDate [DATE] NOT NULL
 IEPServicingEducationOrganizationId [BIGINT] NOT NULL
-StudentIEPAssociationID [NVARCHAR](1024) NOT NULL
-StudentUSI [INT] NOT NULL
-CreateDate [DATETIME] NOT NULL
-LastModifiedDate [DATETIME] NOT NULL
-Id [UNIQUEIDENTIFIER] NOT NULL
-Primary Keys:
-IEPFinalizedDate
-IEPServicingEducationOrganizationId
-StudentIEPAssociationID
-StudentUSI
-sedm.StudentIEPDisability
-IEPFinalizedDate [DATE] NOT NULL
-IEPServicingEducationOrganizationId [BIGINT] NOT NULL
-StudentIEPAssociationID [NVARCHAR](1024) NOT NULL
 StudentUSI [INT] NOT NULL
 DisabilityDescriptorId [INT] NOT NULL
 DisabilityDeterminationSourceTypeDescriptorId [INT] NULL
@@ -19242,23 +19206,28 @@
 OrderOfDisability [INT] NULL
 CreateDate [DATETIME] NOT NULL
 Primary Keys:
-IEPFinalizedDate
 IEPServicingEducationOrganizationId
-StudentIEPAssociationID
 StudentUSI
 DisabilityDescriptorId
+sedm.StudentIEPDisability
+IEPServicingEducationOrganizationId [BIGINT] NOT NULL
+StudentUSI [INT] NOT NULL
+IEPFinalizedDate [DATE] NOT NULL
+StudentIEPAssociationID [NVARCHAR](1024) NOT NULL
+CreateDate [DATETIME] NOT NULL
+LastModifiedDate [DATETIME] NOT NULL
+Id [UNIQUEIDENTIFIER] NOT NULL
+Primary Keys:
+IEPServicingEducationOrganizationId
+StudentUSI
 sedm.StudentIEPDisabilityDesignation
-IEPFinalizedDate [DATE] NOT NULL
 IEPServicingEducationOrganizationId [BIGINT] NOT NULL
-StudentIEPAssociationID [NVARCHAR](1024) NOT NULL
 StudentUSI [INT] NOT NULL
 DisabilityDescriptorId [INT] NOT NULL
 DisabilityDesignationDescriptorId [INT] NOT NULL
 CreateDate [DATETIME] NOT NULL
 Primary Keys:
-IEPFinalizedDate
 IEPServicingEducationOrganizationId
-StudentIEPAssociationID
 StudentUSI
 DisabilityDescriptorId
 DisabilityDesignationDescriptorId
@@ -19334,7 +19303,10 @@
     <t>A unique identifier assigned by the provider of IEP services.</t>
   </si>
   <si>
-    <t>IEPGoalID [NVARCHAR](30)</t>
+    <t>max length: 256</t>
+  </si>
+  <si>
+    <t>IEPGoalID [NVARCHAR](256)</t>
   </si>
   <si>
     <t>IEPGoalDetails</t>
@@ -34680,18 +34652,18 @@
         <v>2606</v>
       </c>
       <c r="D922" t="s">
-        <v>2733</v>
+        <v>3227</v>
       </c>
       <c r="G922" t="s">
-        <v>3227</v>
+        <v>3228</v>
       </c>
     </row>
     <row r="923">
       <c r="A923" t="s">
-        <v>3228</v>
+        <v>3229</v>
       </c>
       <c r="B923" t="s">
-        <v>3229</v>
+        <v>3230</v>
       </c>
       <c r="C923" t="s">
         <v>2606</v>
@@ -34700,15 +34672,15 @@
         <v>3012</v>
       </c>
       <c r="G923" t="s">
-        <v>3230</v>
+        <v>3231</v>
       </c>
     </row>
     <row r="924">
       <c r="A924" t="s">
-        <v>3231</v>
+        <v>3232</v>
       </c>
       <c r="B924" t="s">
-        <v>3232</v>
+        <v>3233</v>
       </c>
       <c r="C924" t="s">
         <v>2606</v>
@@ -34717,7 +34689,7 @@
         <v>2615</v>
       </c>
       <c r="G924" t="s">
-        <v>3233</v>
+        <v>3234</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Reworked extension to make IEP a domain enttity and move other domain entities to associations.
</commit_message>
<xml_diff>
--- a/MetaEdOutput/Documentation/Ed-Fi-Handbook/Ed-Fi-Handbook.xlsx
+++ b/MetaEdOutput/Documentation/Ed-Fi-Handbook/Ed-Fi-Handbook.xlsx
@@ -3614,8 +3614,8 @@
 OrderOfDisability (optional)
 Used By:
 StudentEducationOrganizationAssociation.Disability (as optional collection)
+StudentIEPDisability.Disability (as required collection)
 StudentSpecialEducationProgramAssociation.Disability (as optional collection)
-StudentIEPDisability.Disability (as required collection)
 Disability.Disability (as identity)</t>
   </si>
   <si>
@@ -4230,9 +4230,9 @@
 PrimaryProvider (optional)
 Staff (identity)
 Used By:
+StudentIEPServiceDelivery.ServiceProvider (as optional collection)
 StudentSpecialEducationProgramAssociation.ServiceProvider (as optional collection)
-SpecialEducationProgramService.ServiceProvider (as optional collection)
-IEPServiceDelivery.ServiceProvider (as optional)</t>
+SpecialEducationProgramService.ServiceProvider (as optional collection)</t>
   </si>
   <si>
     <t>SpecialEducationProgramService</t>
@@ -6298,10 +6298,10 @@
   <si>
     <t>Used By:
 StudentAssessmentRegistrationBatteryPartAssociation.Accommodation (as optional collection)
+StudentIEPAccommodation.Accommodation (as required collection)
 StudentAssessment.Accommodation (as optional collection)
 StudentAssessmentRegistration.Accommodation (as optional collection)
-StudentEducationOrganizationAssessmentAccommodation.Accommodation (as optional collection)
-StudentIEPAccommodation.Accommodation (as required collection)</t>
+StudentEducationOrganizationAssessmentAccommodation.Accommodation (as optional collection)</t>
   </si>
   <si>
     <t xml:space="preserve">edfi.AccommodationDescriptor
@@ -7219,8 +7219,8 @@
   <si>
     <t>Used By:
 StudentEducationOrganizationAssociation.Disability (as optional collection)
+StudentIEPDisability.Disability (as required collection)
 StudentSpecialEducationProgramAssociation.Disability (as optional collection)
-StudentIEPDisability.Disability (as required collection)
 Disability.Disability (as identity)</t>
   </si>
   <si>
@@ -8988,7 +8988,7 @@
   <si>
     <t>Used By:
 GeneralStudentProgramAssociation.ReasonExited (as optional)
-StudentIEPAssociation.ReasonExited (as optional)</t>
+StudentIEP.ReasonExited (as optional)</t>
   </si>
   <si>
     <t xml:space="preserve">edfi.ReasonExitedDescriptor
@@ -9474,8 +9474,8 @@
   </si>
   <si>
     <t>Used By:
-StudentIEPAssociation.SpecialEducationSetting (as optional)
-StudentSpecialEducationProgramAssociation.SpecialEducationSetting (as optional)</t>
+StudentSpecialEducationProgramAssociation.SpecialEducationSetting (as optional)
+StudentIEP.SpecialEducationSetting (as optional)</t>
   </si>
   <si>
     <t xml:space="preserve">edfi.SpecialEducationSettingDescriptor
@@ -11871,7 +11871,9 @@
 StudentSpecialEducationProgramEligibilityAssociation.EducationOrganization (as identity)
 SurveyResponseEducationOrganizationTargetAssociation.EducationOrganization (as identity)
 SurveySectionResponseEducationOrganizationTargetAssociation.EducationOrganization (as identity)
-StudentIEPAssociation.EducationOrganization (as identity)
+IEPServicePrescription.EducationOrganization (as optional)
+StudentIEPAccommodation.EducationOrganization (as identity)
+StudentIEPDisability.EducationOrganization (as identity)
 AdministrationPointOfContact.EducationOrganization (as identity)
 ContentStandard.EducationOrganization (as optional)
 DualCredit.EducationOrganization (as optional)
@@ -11902,9 +11904,7 @@
 StudentTransportation.EducationOrganization (as identity)
 Survey.EducationOrganization (as optional)
 IDEAEvent.EducationOrganization (as identity)
-IEPServicePrescription.EducationOrganization (as optional)
-StudentIEPAccommodation.EducationOrganization (as identity)
-StudentIEPDisability.EducationOrganization (as identity)
+StudentIEP.EducationOrganization (as identity)
 OrganizationDepartment.EducationOrganization (as optional)</t>
   </si>
   <si>
@@ -14290,6 +14290,7 @@
 StaffSectionAssociation.Staff (as identity)
 SurveyResponseStaffTargetAssociation.Staff (as identity)
 SurveySectionResponseStaffTargetAssociation.Staff (as identity)
+IEPServicePrescription.Staff (as optional)
 SurveyResponderChoice.Staff (as required)
 ServiceProvider.Staff (as identity)
 CourseTranscript.Staff (as optional)
@@ -14300,9 +14301,7 @@
 SectionAttendanceTakenEvent.Staff (as optional)
 StaffAbsenceEvent.Staff (as identity)
 StaffLeave.Staff (as identity)
-StudentProgramEvaluation.Staff (as optional)
-IEPServiceDelivery.Staff (as optional)
-IEPServicePrescription.Staff (as optional)</t>
+StudentProgramEvaluation.Staff (as optional)</t>
   </si>
   <si>
     <t xml:space="preserve">edfi.Staff
@@ -14625,7 +14624,11 @@
 StudentSchoolAssociation.Student (as identity)
 StudentSectionAssociation.Student (as identity)
 StudentSpecialEducationProgramEligibilityAssociation.Student (as identity)
-StudentIEPAssociation.Student (as identity)
+StudentIEPGoal.Student (as identity)
+StudentIEPServiceDelivery.Student (as identity)
+IEPServicePrescription.Student (as identity)
+StudentIEPAccommodation.Student (as identity)
+StudentIEPDisability.Student (as identity)
 SurveyResponderChoice.Student (as required)
 DisciplineAction.Student (as identity)
 PostSecondaryEvent.Student (as identity)
@@ -14644,11 +14647,7 @@
 StudentSectionAttendanceEvent.Student (as identity)
 StudentTransportation.Student (as identity)
 IDEAEvent.Student (as identity)
-IEPGoal.Student (as identity)
-IEPServiceDelivery.Student (as identity)
-IEPServicePrescription.Student (as identity)
-StudentIEPAccommodation.Student (as identity)
-StudentIEPDisability.Student (as identity)</t>
+StudentIEP.Student (as identity)</t>
   </si>
   <si>
     <t xml:space="preserve">edfi.Student
@@ -18471,7 +18470,800 @@
     <t>PublicationYear [SMALLINT]</t>
   </si>
   <si>
-    <t>StudentIEPAssociation (SEDM)</t>
+    <t>StudentIEPGoal (SEDM)</t>
+  </si>
+  <si>
+    <t>A goal prescribed to a student as part of their IEP.</t>
+  </si>
+  <si>
+    <t>Contains:
+GoalAchievementPeriodBeginDate (optional)
+GoalAchievementPeriodEndDate (optional)
+IDEAEvent (optional collection)
+IEPGoal (required)
+IEPGoalDetails (required)
+IEPGoalID (identity)
+Student (identity)
+StudentIEP (identity)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sedm.StudentIEPGoal
+IEPFinalizedDate [DATE] NOT NULL
+IEPGoalID [NVARCHAR](256) NOT NULL
+IEPServicingEducationOrganizationId [BIGINT] NOT NULL
+StudentIEPAssociationID [NVARCHAR](1024) NOT NULL
+StudentUSI [INT] NOT NULL
+GoalAchievementPeriodBeginDate [DATE] NULL
+GoalAchievementPeriodEndDate [DATE] NULL
+IEPGoalDescriptorId [INT] NOT NULL
+IEPGoalDetails [NVARCHAR](2048) NOT NULL
+CreateDate [DATETIME] NOT NULL
+LastModifiedDate [DATETIME] NOT NULL
+Id [UNIQUEIDENTIFIER] NOT NULL
+Primary Keys:
+IEPFinalizedDate
+IEPGoalID
+IEPServicingEducationOrganizationId
+StudentIEPAssociationID
+StudentUSI
+sedm.StudentIEPGoalIDEAEvent
+IEPFinalizedDate [DATE] NOT NULL
+IEPGoalID [NVARCHAR](256) NOT NULL
+IEPServicingEducationOrganizationId [BIGINT] NOT NULL
+StudentIEPAssociationID [NVARCHAR](1024) NOT NULL
+StudentUSI [INT] NOT NULL
+EducationOrganizationId [BIGINT] NOT NULL
+IDEAEventDescriptorId [INT] NOT NULL
+IDEAEventID [NVARCHAR](1024) NOT NULL
+CreateDate [DATETIME] NOT NULL
+Primary Keys:
+IEPFinalizedDate
+IEPGoalID
+IEPServicingEducationOrganizationId
+StudentIEPAssociationID
+StudentUSI
+EducationOrganizationId
+IDEAEventDescriptorId
+IDEAEventID
+</t>
+  </si>
+  <si>
+    <t>StudentIEPServiceDelivery (SEDM)</t>
+  </si>
+  <si>
+    <t>Services delivered to a student as prescribed by their IEP.</t>
+  </si>
+  <si>
+    <t>Contains:
+ExternalServiceProvider (optional collection)
+IDEAEvent (optional collection)
+IEPServiceDeliveryID (identity)
+IEPServicePrescription (optional)
+ServiceDelivery (identity)
+ServiceDeliveryDate (identity)
+ServiceProvider (optional collection)
+ServiceProviderType (optional)
+Student (identity)
+StudentIEP (identity)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sedm.StudentIEPServiceDelivery
+IEPFinalizedDate [DATE] NOT NULL
+IEPServiceDeliveryID [NVARCHAR](1024) NOT NULL
+IEPServicingEducationOrganizationId [BIGINT] NOT NULL
+ServiceDeliveryDate [DATE] NOT NULL
+ServiceDeliveryDescriptorId [INT] NOT NULL
+StudentIEPAssociationID [NVARCHAR](1024) NOT NULL
+StudentUSI [INT] NOT NULL
+ServicePrescriptionDate [DATE] NULL
+ServicePrescriptionDescriptorId [INT] NULL
+ServiceProviderTypeDescriptorId [INT] NULL
+CreateDate [DATETIME] NOT NULL
+LastModifiedDate [DATETIME] NOT NULL
+Id [UNIQUEIDENTIFIER] NOT NULL
+Primary Keys:
+IEPFinalizedDate
+IEPServiceDeliveryID
+IEPServicingEducationOrganizationId
+ServiceDeliveryDate
+ServiceDeliveryDescriptorId
+StudentIEPAssociationID
+StudentUSI
+sedm.StudentIEPServiceDeliveryExternalServiceProvider
+IEPFinalizedDate [DATE] NOT NULL
+IEPServiceDeliveryID [NVARCHAR](1024) NOT NULL
+IEPServicingEducationOrganizationId [BIGINT] NOT NULL
+ServiceDeliveryDate [DATE] NOT NULL
+ServiceDeliveryDescriptorId [INT] NOT NULL
+StudentIEPAssociationID [NVARCHAR](1024) NOT NULL
+StudentUSI [INT] NOT NULL
+ProviderCode [NVARCHAR](1024) NOT NULL
+ProviderFirstName [NVARCHAR](1024) NOT NULL
+ProviderLastSurname [NVARCHAR](1024) NOT NULL
+PrimaryProvider [BIT] NULL
+ProviderMiddleName [NVARCHAR](1024) NULL
+CreateDate [DATETIME] NOT NULL
+Primary Keys:
+IEPFinalizedDate
+IEPServiceDeliveryID
+IEPServicingEducationOrganizationId
+ServiceDeliveryDate
+ServiceDeliveryDescriptorId
+StudentIEPAssociationID
+StudentUSI
+ProviderCode
+ProviderFirstName
+ProviderLastSurname
+sedm.StudentIEPServiceDeliveryIDEAEvent
+IEPFinalizedDate [DATE] NOT NULL
+IEPServiceDeliveryID [NVARCHAR](1024) NOT NULL
+IEPServicingEducationOrganizationId [BIGINT] NOT NULL
+ServiceDeliveryDate [DATE] NOT NULL
+ServiceDeliveryDescriptorId [INT] NOT NULL
+StudentIEPAssociationID [NVARCHAR](1024) NOT NULL
+StudentUSI [INT] NOT NULL
+EducationOrganizationId [BIGINT] NOT NULL
+IDEAEventDescriptorId [INT] NOT NULL
+IDEAEventID [NVARCHAR](1024) NOT NULL
+CreateDate [DATETIME] NOT NULL
+Primary Keys:
+IEPFinalizedDate
+IEPServiceDeliveryID
+IEPServicingEducationOrganizationId
+ServiceDeliveryDate
+ServiceDeliveryDescriptorId
+StudentIEPAssociationID
+StudentUSI
+EducationOrganizationId
+IDEAEventDescriptorId
+IDEAEventID
+sedm.StudentIEPServiceDeliveryServiceProvider
+IEPFinalizedDate [DATE] NOT NULL
+IEPServiceDeliveryID [NVARCHAR](1024) NOT NULL
+IEPServicingEducationOrganizationId [BIGINT] NOT NULL
+ServiceDeliveryDate [DATE] NOT NULL
+ServiceDeliveryDescriptorId [INT] NOT NULL
+StudentIEPAssociationID [NVARCHAR](1024) NOT NULL
+StudentUSI [INT] NOT NULL
+StaffUSI [INT] NOT NULL
+PrimaryProvider [BIT] NULL
+CreateDate [DATETIME] NOT NULL
+Primary Keys:
+IEPFinalizedDate
+IEPServiceDeliveryID
+IEPServicingEducationOrganizationId
+ServiceDeliveryDate
+ServiceDeliveryDescriptorId
+StudentIEPAssociationID
+StudentUSI
+StaffUSI
+</t>
+  </si>
+  <si>
+    <t>IEPServicePrescription (SEDM)</t>
+  </si>
+  <si>
+    <t>The service prescribed to a student as part of their IEP.</t>
+  </si>
+  <si>
+    <t>Contains:
+BeginDate (required)
+DurationMinutes (required)
+DurationPeriod (required)
+EducationOrganization (optional)
+EndDate (optional)
+FrequencyPeriod (required)
+FrequencyValue (required)
+IDEAEvent (optional collection)
+ServiceLocationType (required)
+ServicePrescription (identity)
+ServicePrescriptionDate (identity)
+Staff (optional)
+Student (identity)
+StudentIEP (identity)
+Used By:
+StudentIEPServiceDelivery.IEPServicePrescription (as optional)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sedm.IEPServicePrescription
+IEPFinalizedDate [DATE] NOT NULL
+IEPServicingEducationOrganizationId [BIGINT] NOT NULL
+ServicePrescriptionDate [DATE] NOT NULL
+ServicePrescriptionDescriptorId [INT] NOT NULL
+StudentIEPAssociationID [NVARCHAR](1024) NOT NULL
+StudentUSI [INT] NOT NULL
+BeginDate [DATE] NOT NULL
+DurationMinutes [DECIMAL](5, 2) NOT NULL
+DurationPeriodDescriptorId [INT] NOT NULL
+EndDate [DATE] NULL
+FrequencyPeriodDescriptorId [INT] NOT NULL
+FrequencyValue [DECIMAL](5, 2) NOT NULL
+ServiceLocationTypeDescriptorId [INT] NOT NULL
+ServiceProvidingEducationOrganizationId [BIGINT] NULL
+StaffUSI [INT] NULL
+CreateDate [DATETIME] NOT NULL
+LastModifiedDate [DATETIME] NOT NULL
+Id [UNIQUEIDENTIFIER] NOT NULL
+Primary Keys:
+IEPFinalizedDate
+IEPServicingEducationOrganizationId
+ServicePrescriptionDate
+ServicePrescriptionDescriptorId
+StudentIEPAssociationID
+StudentUSI
+sedm.IEPServicePrescriptionIDEAEvent
+IEPFinalizedDate [DATE] NOT NULL
+IEPServicingEducationOrganizationId [BIGINT] NOT NULL
+ServicePrescriptionDate [DATE] NOT NULL
+ServicePrescriptionDescriptorId [INT] NOT NULL
+StudentIEPAssociationID [NVARCHAR](1024) NOT NULL
+StudentUSI [INT] NOT NULL
+EducationOrganizationId [BIGINT] NOT NULL
+IDEAEventDescriptorId [INT] NOT NULL
+IDEAEventID [NVARCHAR](1024) NOT NULL
+CreateDate [DATETIME] NOT NULL
+Primary Keys:
+IEPFinalizedDate
+IEPServicingEducationOrganizationId
+ServicePrescriptionDate
+ServicePrescriptionDescriptorId
+StudentIEPAssociationID
+StudentUSI
+EducationOrganizationId
+IDEAEventDescriptorId
+IDEAEventID
+</t>
+  </si>
+  <si>
+    <t>StudentIEPAccommodation (SEDM)</t>
+  </si>
+  <si>
+    <t>The accommodations prescribed to a student as part of their IEP.</t>
+  </si>
+  <si>
+    <t>Contains:
+Accommodation (required collection)
+EducationOrganization (identity)
+Student (identity)
+StudentIEP (identity)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sedm.StudentIEPAccommodation
+IEPFinalizedDate [DATE] NOT NULL
+IEPServicingEducationOrganizationId [BIGINT] NOT NULL
+StudentIEPAssociationID [NVARCHAR](1024) NOT NULL
+StudentUSI [INT] NOT NULL
+AccommodationDescriptorId [INT] NOT NULL
+CreateDate [DATETIME] NOT NULL
+Primary Keys:
+IEPFinalizedDate
+IEPServicingEducationOrganizationId
+StudentIEPAssociationID
+StudentUSI
+AccommodationDescriptorId
+sedm.StudentIEPAccommodation
+IEPFinalizedDate [DATE] NOT NULL
+IEPServicingEducationOrganizationId [BIGINT] NOT NULL
+StudentIEPAssociationID [NVARCHAR](1024) NOT NULL
+StudentUSI [INT] NOT NULL
+CreateDate [DATETIME] NOT NULL
+LastModifiedDate [DATETIME] NOT NULL
+Id [UNIQUEIDENTIFIER] NOT NULL
+Primary Keys:
+IEPFinalizedDate
+IEPServicingEducationOrganizationId
+StudentIEPAssociationID
+StudentUSI
+</t>
+  </si>
+  <si>
+    <t>StudentIEPDisability (SEDM)</t>
+  </si>
+  <si>
+    <t>The disabilities prescribed to a student as part of their IEP.</t>
+  </si>
+  <si>
+    <t>Contains:
+Disability (required collection)
+EducationOrganization (identity)
+Student (identity)
+StudentIEP (identity)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sedm.StudentIEPDisability
+IEPFinalizedDate [DATE] NOT NULL
+IEPServicingEducationOrganizationId [BIGINT] NOT NULL
+StudentIEPAssociationID [NVARCHAR](1024) NOT NULL
+StudentUSI [INT] NOT NULL
+CreateDate [DATETIME] NOT NULL
+LastModifiedDate [DATETIME] NOT NULL
+Id [UNIQUEIDENTIFIER] NOT NULL
+Primary Keys:
+IEPFinalizedDate
+IEPServicingEducationOrganizationId
+StudentIEPAssociationID
+StudentUSI
+sedm.StudentIEPDisability
+IEPFinalizedDate [DATE] NOT NULL
+IEPServicingEducationOrganizationId [BIGINT] NOT NULL
+StudentIEPAssociationID [NVARCHAR](1024) NOT NULL
+StudentUSI [INT] NOT NULL
+DisabilityDescriptorId [INT] NOT NULL
+DisabilityDeterminationSourceTypeDescriptorId [INT] NULL
+DisabilityDiagnosis [NVARCHAR](80) NULL
+OrderOfDisability [INT] NULL
+CreateDate [DATETIME] NOT NULL
+Primary Keys:
+IEPFinalizedDate
+IEPServicingEducationOrganizationId
+StudentIEPAssociationID
+StudentUSI
+DisabilityDescriptorId
+sedm.StudentIEPDisabilityDesignation
+IEPFinalizedDate [DATE] NOT NULL
+IEPServicingEducationOrganizationId [BIGINT] NOT NULL
+StudentIEPAssociationID [NVARCHAR](1024) NOT NULL
+StudentUSI [INT] NOT NULL
+DisabilityDescriptorId [INT] NOT NULL
+DisabilityDesignationDescriptorId [INT] NOT NULL
+CreateDate [DATETIME] NOT NULL
+Primary Keys:
+IEPFinalizedDate
+IEPServicingEducationOrganizationId
+StudentIEPAssociationID
+StudentUSI
+DisabilityDescriptorId
+DisabilityDesignationDescriptorId
+</t>
+  </si>
+  <si>
+    <t>Primary External Service Provider.</t>
+  </si>
+  <si>
+    <t>Used By:
+ExternalServiceProvider.PrimaryProvider (as optional)</t>
+  </si>
+  <si>
+    <t>Used By:
+StudentIEP.MedicallyFragile (as optional)</t>
+  </si>
+  <si>
+    <t>Used By:
+StudentIEP.MultiplyDisabled (as optional)</t>
+  </si>
+  <si>
+    <t>ExternalServiceProvider (SEDM)</t>
+  </si>
+  <si>
+    <t>A service provider that is external to the education organization and is not present in the Staffs resource.</t>
+  </si>
+  <si>
+    <t>Contains:
+PrimaryProvider (optional)
+ProviderCode (identity)
+ProviderFirstName (identity)
+ProviderLastSurname (identity)
+ProviderMiddleName (optional)
+Used By:
+StudentIEPServiceDelivery.ExternalServiceProvider (as optional collection)</t>
+  </si>
+  <si>
+    <t>GoalAchievementPeriodBeginDate</t>
+  </si>
+  <si>
+    <t>The first date of the period assigned for achieving the stated goal.</t>
+  </si>
+  <si>
+    <t>Used By:
+StudentIEPGoal.GoalAchievementPeriodBeginDate (as optional)</t>
+  </si>
+  <si>
+    <t>GoalAchievementPeriodBeginDate [DATE]</t>
+  </si>
+  <si>
+    <t>GoalAchievementPeriodEndDate</t>
+  </si>
+  <si>
+    <t>The last date of the period assigned for achieving the stated goal.</t>
+  </si>
+  <si>
+    <t>Used By:
+StudentIEPGoal.GoalAchievementPeriodEndDate (as optional)</t>
+  </si>
+  <si>
+    <t>GoalAchievementPeriodEndDate [DATE]</t>
+  </si>
+  <si>
+    <t>ServiceDeliveryDate</t>
+  </si>
+  <si>
+    <t>The date when prescribed services were delivered for a student.</t>
+  </si>
+  <si>
+    <t>Used By:
+StudentIEPServiceDelivery.ServiceDeliveryDate (as identity)</t>
+  </si>
+  <si>
+    <t>ServiceDeliveryDate [DATE]</t>
+  </si>
+  <si>
+    <t>ServicePrescriptionDate</t>
+  </si>
+  <si>
+    <t>The date the service was prescribed.</t>
+  </si>
+  <si>
+    <t>Used By:
+IEPServicePrescription.ServicePrescriptionDate (as identity)</t>
+  </si>
+  <si>
+    <t>ServicePrescriptionDate [DATE]</t>
+  </si>
+  <si>
+    <t>BeginDate (IEPServicePrescription)</t>
+  </si>
+  <si>
+    <t>The effective date when service is to begin.</t>
+  </si>
+  <si>
+    <t>Used By:
+IEPServicePrescription.BeginDate (as required)</t>
+  </si>
+  <si>
+    <t>EndDate (IEPServicePrescription)</t>
+  </si>
+  <si>
+    <t>The effective date when the prescribed service ended.</t>
+  </si>
+  <si>
+    <t>Used By:
+IEPServicePrescription.EndDate (as optional)</t>
+  </si>
+  <si>
+    <t>EventBeginDate</t>
+  </si>
+  <si>
+    <t>The date when the IDEA related event started.</t>
+  </si>
+  <si>
+    <t>Used By:
+IDEAEvent.EventBeginDate (as required)</t>
+  </si>
+  <si>
+    <t>EventBeginDate [DATE]</t>
+  </si>
+  <si>
+    <t>EventEndDate</t>
+  </si>
+  <si>
+    <t>The date when the IDEA event concluded.</t>
+  </si>
+  <si>
+    <t>Used By:
+IDEAEvent.EventEndDate (as required)</t>
+  </si>
+  <si>
+    <t>EventEndDate [DATE]</t>
+  </si>
+  <si>
+    <t>IEPFinalizedDate</t>
+  </si>
+  <si>
+    <t>The date the most recent IEP was finalized.  Note: Date interpretation may vary. Ed-Fi recommends inclusive dates, but states may define dates as inclusive or exclusive. For calculations, align with local guidelines.</t>
+  </si>
+  <si>
+    <t>Used By:
+StudentIEP.IEPFinalizedDate (as identity)</t>
+  </si>
+  <si>
+    <t>IEPFinalizedDate [DATE]</t>
+  </si>
+  <si>
+    <t>The effective start date of the most recent IEP.  Note: Date interpretation may vary. Ed-Fi recommends inclusive dates, but states may define dates as inclusive or exclusive. For calculations, align with local guidelines.</t>
+  </si>
+  <si>
+    <t>Used By:
+StudentIEP.IEPBeginDate (as required)</t>
+  </si>
+  <si>
+    <t>The effective end date of the most recent IEP.  Note: Date interpretation may vary. Ed-Fi recommends inclusive dates, but states may define dates as inclusive or exclusive. For calculations, align with local guidelines.</t>
+  </si>
+  <si>
+    <t>Used By:
+StudentIEP.IEPEndDate (as required)</t>
+  </si>
+  <si>
+    <t>IEPAmendedDate</t>
+  </si>
+  <si>
+    <t>The date when the most recent IEP was last amended, if any.  Note: Date interpretation may vary. Ed-Fi recommends inclusive dates, but states may define dates as inclusive or exclusive. For calculations, align with local guidelines.</t>
+  </si>
+  <si>
+    <t>Used By:
+StudentIEP.IEPAmendedDate (as optional)</t>
+  </si>
+  <si>
+    <t>IEPAmendedDate [DATE]</t>
+  </si>
+  <si>
+    <t>DurationMinutes</t>
+  </si>
+  <si>
+    <t>The length of time for the prescribed service in minutes.</t>
+  </si>
+  <si>
+    <t>DurationMinutes [DECIMAL](5, 2)</t>
+  </si>
+  <si>
+    <t>FrequencyValue</t>
+  </si>
+  <si>
+    <t>The number of times the prescribed service is to be provided within the specified duration period.</t>
+  </si>
+  <si>
+    <t>FrequencyValue [DECIMAL](5, 2)</t>
+  </si>
+  <si>
+    <t>DurationPeriod (SEDM)</t>
+  </si>
+  <si>
+    <t>The frequency period for the prescribed service duration. Examples include: Per Session, Per Week, Per Month.</t>
+  </si>
+  <si>
+    <t>Used By:
+IEPServicePrescription.DurationPeriod (as required)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sedm.DurationPeriodDescriptor
+DurationPeriodDescriptorId [INT] NOT NULL
+Primary Keys:
+DurationPeriodDescriptorId
+</t>
+  </si>
+  <si>
+    <t>EventCompliance (SEDM)</t>
+  </si>
+  <si>
+    <t>The policy or law for which an event is compliant.</t>
+  </si>
+  <si>
+    <t>Used By:
+IDEAEvent.EventCompliance (as optional)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sedm.EventComplianceDescriptor
+EventComplianceDescriptorId [INT] NOT NULL
+Primary Keys:
+EventComplianceDescriptorId
+</t>
+  </si>
+  <si>
+    <t>EventReason (SEDM)</t>
+  </si>
+  <si>
+    <t>Reason the event occured.</t>
+  </si>
+  <si>
+    <t>Used By:
+IDEAEvent.EventReason (as optional)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sedm.EventReasonDescriptor
+EventReasonDescriptorId [INT] NOT NULL
+Primary Keys:
+EventReasonDescriptorId
+</t>
+  </si>
+  <si>
+    <t>FrequencyPeriod (SEDM)</t>
+  </si>
+  <si>
+    <t>The frequency period for the prescribed service. Examples include: Session, Week, Month.</t>
+  </si>
+  <si>
+    <t>Used By:
+IEPServicePrescription.FrequencyPeriod (as required)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sedm.FrequencyPeriodDescriptor
+FrequencyPeriodDescriptorId [INT] NOT NULL
+Primary Keys:
+FrequencyPeriodDescriptorId
+</t>
+  </si>
+  <si>
+    <t>IDEAEvent (SEDM)</t>
+  </si>
+  <si>
+    <t>IDEA event type. Examples: Referral for Evaluation, IEP Approved, Parental COnsent Given, Evaluation Complete.</t>
+  </si>
+  <si>
+    <t>Used By:
+IDEAEvent.IDEAEvent (as identity)
+StudentIEPGoal.IDEAEvent (as optional collection)
+StudentIEPServiceDelivery.IDEAEvent (as optional collection)
+IEPServicePrescription.IDEAEvent (as optional collection)
+StudentIEP.IDEAEvent (as optional collection)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sedm.IDEAEventDescriptor
+IDEAEventDescriptorId [INT] NOT NULL
+Primary Keys:
+IDEAEventDescriptorId
+</t>
+  </si>
+  <si>
+    <t>IEPGoal (SEDM)</t>
+  </si>
+  <si>
+    <t>A focused goal for an IEP.</t>
+  </si>
+  <si>
+    <t>Used By:
+StudentIEPGoal.IEPGoal (as required)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sedm.IEPGoalDescriptor
+IEPGoalDescriptorId [INT] NOT NULL
+Primary Keys:
+IEPGoalDescriptorId
+</t>
+  </si>
+  <si>
+    <t>IEPStatus (SEDM)</t>
+  </si>
+  <si>
+    <t>The current status of the student IEP.</t>
+  </si>
+  <si>
+    <t>Used By:
+StudentIEP.IEPStatus (as required)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sedm.IEPStatusDescriptor
+IEPStatusDescriptorId [INT] NOT NULL
+Primary Keys:
+IEPStatusDescriptorId
+</t>
+  </si>
+  <si>
+    <t>ServiceCompliance (SEDM)</t>
+  </si>
+  <si>
+    <t>The policy or law for which a prescribed service is compliant.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sedm.ServiceComplianceDescriptor
+ServiceComplianceDescriptorId [INT] NOT NULL
+Primary Keys:
+ServiceComplianceDescriptorId
+</t>
+  </si>
+  <si>
+    <t>ServiceDelivery (SEDM)</t>
+  </si>
+  <si>
+    <t>The type of service provided to a student.</t>
+  </si>
+  <si>
+    <t>Used By:
+StudentIEPServiceDelivery.ServiceDelivery (as identity)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sedm.ServiceDeliveryDescriptor
+ServiceDeliveryDescriptorId [INT] NOT NULL
+Primary Keys:
+ServiceDeliveryDescriptorId
+</t>
+  </si>
+  <si>
+    <t>ServiceLocationType (SEDM)</t>
+  </si>
+  <si>
+    <t>The location type where the prescribed service is to be provided. Examples include: Home, Hospital, School.</t>
+  </si>
+  <si>
+    <t>Used By:
+IEPServicePrescription.ServiceLocationType (as required)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sedm.ServiceLocationTypeDescriptor
+ServiceLocationTypeDescriptorId [INT] NOT NULL
+Primary Keys:
+ServiceLocationTypeDescriptorId
+</t>
+  </si>
+  <si>
+    <t>ServicePrescription (SEDM)</t>
+  </si>
+  <si>
+    <t>The type of service prescribed.</t>
+  </si>
+  <si>
+    <t>Used By:
+IEPServicePrescription.ServicePrescription (as identity)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sedm.ServicePrescriptionDescriptor
+ServicePrescriptionDescriptorId [INT] NOT NULL
+Primary Keys:
+ServicePrescriptionDescriptorId
+</t>
+  </si>
+  <si>
+    <t>ServiceProviderType (SEDM)</t>
+  </si>
+  <si>
+    <t>Indicates service provider type, including specialist, internal staff, external staff, etc.</t>
+  </si>
+  <si>
+    <t>Used By:
+StudentIEPServiceDelivery.ServiceProviderType (as optional)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sedm.ServiceProviderTypeDescriptor
+ServiceProviderTypeDescriptorId [INT] NOT NULL
+Primary Keys:
+ServiceProviderTypeDescriptorId
+</t>
+  </si>
+  <si>
+    <t>ServiceReason (SEDM)</t>
+  </si>
+  <si>
+    <t>Reason the service was prescribed. Examples include: Counselor Assigned, IEP Team Determination.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sedm.ServiceReasonDescriptor
+ServiceReasonDescriptorId [INT] NOT NULL
+Primary Keys:
+ServiceReasonDescriptorId
+</t>
+  </si>
+  <si>
+    <t>An IDEA related student event describing status, dates and narrative.</t>
+  </si>
+  <si>
+    <t>Contains:
+EducationOrganization (identity)
+EventBeginDate (required)
+EventCompliance (optional)
+EventEndDate (required)
+EventNarrative (optional)
+EventReason (optional)
+IDEAEvent (identity)
+IDEAEventID (identity)
+Student (identity)
+Used By:
+IDEAEvent.IDEAEvent (as identity)
+StudentIEPGoal.IDEAEvent (as optional collection)
+StudentIEPServiceDelivery.IDEAEvent (as optional collection)
+IEPServicePrescription.IDEAEvent (as optional collection)
+StudentIEP.IDEAEvent (as optional collection)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sedm.IDEAEvent
+EducationOrganizationId [BIGINT] NOT NULL
+IDEAEventDescriptorId [INT] NOT NULL
+IDEAEventID [NVARCHAR](1024) NOT NULL
+StudentUSI [INT] NOT NULL
+EventBeginDate [DATE] NOT NULL
+EventComplianceDescriptorId [INT] NULL
+EventEndDate [DATE] NOT NULL
+EventNarrative [NVARCHAR](2048) NULL
+EventReasonDescriptorId [INT] NULL
+CreateDate [DATETIME] NOT NULL
+LastModifiedDate [DATETIME] NOT NULL
+Id [UNIQUEIDENTIFIER] NOT NULL
+Primary Keys:
+EducationOrganizationId
+IDEAEventDescriptorId
+IDEAEventID
+StudentUSI
+</t>
+  </si>
+  <si>
+    <t>StudentIEP (SEDM)</t>
   </si>
   <si>
     <t>This association describes summary IEP data for a student receiving special education services.</t>
@@ -18494,14 +19286,14 @@
 Student (identity)
 StudentIEPAssociationID (identity)
 Used By:
-IEPGoal.StudentIEPAssociation (as required)
-IEPServiceDelivery.StudentIEPAssociation (as required)
-IEPServicePrescription.StudentIEPAssociation (as required)
-StudentIEPAccommodation.StudentIEPAssociation (as required)
-StudentIEPDisability.StudentIEPAssociation (as required)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sedm.StudentIEPAssociation
+StudentIEPGoal.StudentIEP (as identity)
+StudentIEPServiceDelivery.StudentIEP (as identity)
+IEPServicePrescription.StudentIEP (as identity)
+StudentIEPAccommodation.StudentIEP (as identity)
+StudentIEPDisability.StudentIEP (as identity)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sedm.StudentIEP
 IEPFinalizedDate [DATE] NOT NULL
 IEPServicingEducationOrganizationId [BIGINT] NOT NULL
 StudentIEPAssociationID [NVARCHAR](1024) NOT NULL
@@ -18524,7 +19316,7 @@
 IEPServicingEducationOrganizationId
 StudentIEPAssociationID
 StudentUSI
-sedm.StudentIEPAssociationIDEAEvent
+sedm.StudentIEPIDEAEvent
 IEPFinalizedDate [DATE] NOT NULL
 IEPServicingEducationOrganizationId [BIGINT] NOT NULL
 StudentIEPAssociationID [NVARCHAR](1024) NOT NULL
@@ -18544,694 +19336,88 @@
 </t>
   </si>
   <si>
-    <t>Used By:
-StudentIEPAssociation.MedicallyFragile (as optional)</t>
-  </si>
-  <si>
-    <t>Used By:
-StudentIEPAssociation.MultiplyDisabled (as optional)</t>
-  </si>
-  <si>
-    <t>Primary External Service Provider.</t>
-  </si>
-  <si>
-    <t>Used By:
-ExternalServiceProvider.PrimaryProvider (as optional)</t>
-  </si>
-  <si>
-    <t>ExternalServiceProvider (SEDM)</t>
-  </si>
-  <si>
-    <t>A service provider that is external to the education organization and is not present in the Staffs resource.</t>
-  </si>
-  <si>
-    <t>Contains:
-PrimaryProvider (optional)
-ProviderCode (identity)
-ProviderFirstName (identity)
-ProviderLastSurname (identity)
-ProviderMiddleName (optional)
-Used By:
-IEPServiceDelivery.ExternalServiceProvider (as optional collection)</t>
-  </si>
-  <si>
-    <t>IEPFinalizedDate</t>
-  </si>
-  <si>
-    <t>The date the most recent IEP was finalized.  Note: Date interpretation may vary. Ed-Fi recommends inclusive dates, but states may define dates as inclusive or exclusive. For calculations, align with local guidelines.</t>
-  </si>
-  <si>
-    <t>Used By:
-StudentIEPAssociation.IEPFinalizedDate (as identity)</t>
-  </si>
-  <si>
-    <t>IEPFinalizedDate [DATE]</t>
-  </si>
-  <si>
-    <t>The effective start date of the most recent IEP.  Note: Date interpretation may vary. Ed-Fi recommends inclusive dates, but states may define dates as inclusive or exclusive. For calculations, align with local guidelines.</t>
-  </si>
-  <si>
-    <t>Used By:
-StudentIEPAssociation.IEPBeginDate (as required)</t>
-  </si>
-  <si>
-    <t>The effective end date of the most recent IEP.  Note: Date interpretation may vary. Ed-Fi recommends inclusive dates, but states may define dates as inclusive or exclusive. For calculations, align with local guidelines.</t>
-  </si>
-  <si>
-    <t>Used By:
-StudentIEPAssociation.IEPEndDate (as required)</t>
-  </si>
-  <si>
-    <t>IEPAmendedDate</t>
-  </si>
-  <si>
-    <t>The date when the most recent IEP was last amended, if any.  Note: Date interpretation may vary. Ed-Fi recommends inclusive dates, but states may define dates as inclusive or exclusive. For calculations, align with local guidelines.</t>
-  </si>
-  <si>
-    <t>Used By:
-StudentIEPAssociation.IEPAmendedDate (as optional)</t>
-  </si>
-  <si>
-    <t>IEPAmendedDate [DATE]</t>
-  </si>
-  <si>
-    <t>EventBeginDate</t>
-  </si>
-  <si>
-    <t>The date when the IDEA related event started.</t>
-  </si>
-  <si>
-    <t>Used By:
-IDEAEvent.EventBeginDate (as required)</t>
-  </si>
-  <si>
-    <t>EventBeginDate [DATE]</t>
-  </si>
-  <si>
-    <t>EventEndDate</t>
-  </si>
-  <si>
-    <t>The date when the IDEA event concluded.</t>
-  </si>
-  <si>
-    <t>Used By:
-IDEAEvent.EventEndDate (as required)</t>
-  </si>
-  <si>
-    <t>EventEndDate [DATE]</t>
-  </si>
-  <si>
-    <t>GoalAchievementPeriodBeginDate</t>
-  </si>
-  <si>
-    <t>The first date of the period assigned for achieving the stated goal.</t>
-  </si>
-  <si>
-    <t>Used By:
-IEPGoal.GoalAchievementPeriodBeginDate (as optional)</t>
-  </si>
-  <si>
-    <t>GoalAchievementPeriodBeginDate [DATE]</t>
-  </si>
-  <si>
-    <t>GoalAchievementPeriodEndDate</t>
-  </si>
-  <si>
-    <t>The last date of the period assigned for achieving the stated goal.</t>
-  </si>
-  <si>
-    <t>Used By:
-IEPGoal.GoalAchievementPeriodEndDate (as optional)</t>
-  </si>
-  <si>
-    <t>GoalAchievementPeriodEndDate [DATE]</t>
-  </si>
-  <si>
-    <t>ServiceDeliveryDate</t>
-  </si>
-  <si>
-    <t>The date when prescribed services were delivered for a student.</t>
-  </si>
-  <si>
-    <t>Used By:
-IEPServiceDelivery.ServiceDeliveryDate (as identity)</t>
-  </si>
-  <si>
-    <t>ServiceDeliveryDate [DATE]</t>
-  </si>
-  <si>
-    <t>ServicePrescriptionDate</t>
-  </si>
-  <si>
-    <t>The date the service was prescribed.</t>
-  </si>
-  <si>
-    <t>Used By:
-IEPServicePrescription.ServicePrescriptionDate (as identity)</t>
-  </si>
-  <si>
-    <t>ServicePrescriptionDate [DATE]</t>
-  </si>
-  <si>
-    <t>BeginDate (IEPServicePrescription)</t>
-  </si>
-  <si>
-    <t>The effective date when service is to begin.</t>
-  </si>
-  <si>
-    <t>Used By:
-IEPServicePrescription.BeginDate (as required)</t>
-  </si>
-  <si>
-    <t>EndDate (IEPServicePrescription)</t>
-  </si>
-  <si>
-    <t>The effective date when the prescribed service ended.</t>
-  </si>
-  <si>
-    <t>Used By:
-IEPServicePrescription.EndDate (as optional)</t>
-  </si>
-  <si>
-    <t>DurationMinutes</t>
-  </si>
-  <si>
-    <t>The length of time for the prescribed service in minutes.</t>
-  </si>
-  <si>
-    <t>DurationMinutes [DECIMAL](5, 2)</t>
-  </si>
-  <si>
-    <t>FrequencyValue</t>
-  </si>
-  <si>
-    <t>The number of times the prescribed service is to be provided within the specified duration period.</t>
-  </si>
-  <si>
-    <t>FrequencyValue [DECIMAL](5, 2)</t>
-  </si>
-  <si>
-    <t>DurationPeriod (SEDM)</t>
-  </si>
-  <si>
-    <t>The frequency period for the prescribed service duration. Examples include: Per Session, Per Week, Per Month.</t>
-  </si>
-  <si>
-    <t>Used By:
-IEPServicePrescription.DurationPeriod (as required)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sedm.DurationPeriodDescriptor
-DurationPeriodDescriptorId [INT] NOT NULL
-Primary Keys:
-DurationPeriodDescriptorId
-</t>
-  </si>
-  <si>
-    <t>EventCompliance (SEDM)</t>
-  </si>
-  <si>
-    <t>The policy or law for which an event is compliant.</t>
-  </si>
-  <si>
-    <t>Used By:
-IDEAEvent.EventCompliance (as optional)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sedm.EventComplianceDescriptor
-EventComplianceDescriptorId [INT] NOT NULL
-Primary Keys:
-EventComplianceDescriptorId
-</t>
-  </si>
-  <si>
-    <t>EventReason (SEDM)</t>
-  </si>
-  <si>
-    <t>Reason the event occured.</t>
-  </si>
-  <si>
-    <t>Used By:
-IDEAEvent.EventReason (as optional)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sedm.EventReasonDescriptor
-EventReasonDescriptorId [INT] NOT NULL
-Primary Keys:
-EventReasonDescriptorId
-</t>
-  </si>
-  <si>
-    <t>FrequencyPeriod (SEDM)</t>
-  </si>
-  <si>
-    <t>The frequency period for the prescribed service. Examples include: Session, Week, Month.</t>
-  </si>
-  <si>
-    <t>Used By:
-IEPServicePrescription.FrequencyPeriod (as required)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sedm.FrequencyPeriodDescriptor
-FrequencyPeriodDescriptorId [INT] NOT NULL
-Primary Keys:
-FrequencyPeriodDescriptorId
-</t>
-  </si>
-  <si>
-    <t>IDEAEvent (SEDM)</t>
-  </si>
-  <si>
-    <t>IDEA event type. Examples: Referral for Evaluation, IEP Approved, Parental COnsent Given, Evaluation Complete.</t>
-  </si>
-  <si>
-    <t>Used By:
-IDEAEvent.IDEAEvent (as identity)
-StudentIEPAssociation.IDEAEvent (as optional collection)
-IEPGoal.IDEAEvent (as optional)
-IEPServiceDelivery.IDEAEvent (as optional)
-IEPServicePrescription.IDEAEvent (as optional)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sedm.IDEAEventDescriptor
-IDEAEventDescriptorId [INT] NOT NULL
-Primary Keys:
-IDEAEventDescriptorId
-</t>
-  </si>
-  <si>
-    <t>IEPGoal (SEDM)</t>
-  </si>
-  <si>
-    <t>A focused goal for an IEP.</t>
-  </si>
-  <si>
-    <t>Used By:
-IEPGoal.IEPGoal (as required)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sedm.IEPGoalDescriptor
-IEPGoalDescriptorId [INT] NOT NULL
-Primary Keys:
-IEPGoalDescriptorId
-</t>
-  </si>
-  <si>
-    <t>IEPStatus (SEDM)</t>
-  </si>
-  <si>
-    <t>The current status of the student IEP.</t>
-  </si>
-  <si>
-    <t>Used By:
-StudentIEPAssociation.IEPStatus (as required)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sedm.IEPStatusDescriptor
-IEPStatusDescriptorId [INT] NOT NULL
-Primary Keys:
-IEPStatusDescriptorId
-</t>
-  </si>
-  <si>
-    <t>ServiceCompliance (SEDM)</t>
-  </si>
-  <si>
-    <t>The policy or law for which a prescribed service is compliant.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sedm.ServiceComplianceDescriptor
-ServiceComplianceDescriptorId [INT] NOT NULL
-Primary Keys:
-ServiceComplianceDescriptorId
-</t>
-  </si>
-  <si>
-    <t>ServiceDelivery (SEDM)</t>
-  </si>
-  <si>
-    <t>The type of service provided to a student.</t>
-  </si>
-  <si>
-    <t>Used By:
-IEPServiceDelivery.ServiceDelivery (as identity)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sedm.ServiceDeliveryDescriptor
-ServiceDeliveryDescriptorId [INT] NOT NULL
-Primary Keys:
-ServiceDeliveryDescriptorId
-</t>
-  </si>
-  <si>
-    <t>ServiceLocationType (SEDM)</t>
-  </si>
-  <si>
-    <t>The location type where the prescribed service is to be provided. Examples include: Home, Hospital, School.</t>
-  </si>
-  <si>
-    <t>Used By:
-IEPServicePrescription.ServiceLocationType (as required)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sedm.ServiceLocationTypeDescriptor
-ServiceLocationTypeDescriptorId [INT] NOT NULL
-Primary Keys:
-ServiceLocationTypeDescriptorId
-</t>
-  </si>
-  <si>
-    <t>ServicePrescription (SEDM)</t>
-  </si>
-  <si>
-    <t>The type of service prescribed.</t>
-  </si>
-  <si>
-    <t>Used By:
-IEPServicePrescription.ServicePrescription (as identity)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sedm.ServicePrescriptionDescriptor
-ServicePrescriptionDescriptorId [INT] NOT NULL
-Primary Keys:
-ServicePrescriptionDescriptorId
-</t>
-  </si>
-  <si>
-    <t>ServiceProvider (SEDM)</t>
-  </si>
-  <si>
-    <t>Indicates service provider type, including specialist, internal staff, external staff, etc.</t>
-  </si>
-  <si>
-    <t>Used By:
-StudentSpecialEducationProgramAssociation.ServiceProvider (as optional collection)
-SpecialEducationProgramService.ServiceProvider (as optional collection)
-IEPServiceDelivery.ServiceProvider (as optional)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sedm.ServiceProviderDescriptor
-ServiceProviderDescriptorId [INT] NOT NULL
-Primary Keys:
-ServiceProviderDescriptorId
-</t>
-  </si>
-  <si>
-    <t>ServiceReason (SEDM)</t>
-  </si>
-  <si>
-    <t>Reason the service was prescribed. Examples include: Counselor Assigned, IEP Team Determination.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sedm.ServiceReasonDescriptor
-ServiceReasonDescriptorId [INT] NOT NULL
-Primary Keys:
-ServiceReasonDescriptorId
-</t>
-  </si>
-  <si>
-    <t>An IDEA related student event describing status, dates and narrative.</t>
-  </si>
-  <si>
-    <t>Contains:
-EducationOrganization (identity)
-EventBeginDate (required)
-EventCompliance (optional)
-EventEndDate (required)
-EventNarrative (optional)
-EventReason (optional)
-IDEAEvent (identity)
-IDEAEventID (identity)
-Student (identity)
-Used By:
-IDEAEvent.IDEAEvent (as identity)
-StudentIEPAssociation.IDEAEvent (as optional collection)
-IEPGoal.IDEAEvent (as optional)
-IEPServiceDelivery.IDEAEvent (as optional)
-IEPServicePrescription.IDEAEvent (as optional)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sedm.IDEAEvent
-EducationOrganizationId [BIGINT] NOT NULL
-IDEAEventDescriptorId [INT] NOT NULL
-IDEAEventID [NVARCHAR](1024) NOT NULL
-StudentUSI [INT] NOT NULL
-EventBeginDate [DATE] NOT NULL
-EventComplianceDescriptorId [INT] NULL
-EventEndDate [DATE] NOT NULL
-EventNarrative [NVARCHAR](2048) NULL
-EventReasonDescriptorId [INT] NULL
-CreateDate [DATETIME] NOT NULL
-LastModifiedDate [DATETIME] NOT NULL
-Id [UNIQUEIDENTIFIER] NOT NULL
-Primary Keys:
-EducationOrganizationId
-IDEAEventDescriptorId
-IDEAEventID
-StudentUSI
-</t>
-  </si>
-  <si>
-    <t>A goal prescribed to a student as part of their IEP.</t>
-  </si>
-  <si>
-    <t>Contains:
-GoalAchievementPeriodBeginDate (optional)
-GoalAchievementPeriodEndDate (optional)
-IDEAEvent (optional)
-IEPGoal (required)
-IEPGoalDetails (required)
-IEPGoalID (identity)
-Student (identity)
-StudentIEPAssociation (required)
-Used By:
-IEPGoal.IEPGoal (as required)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sedm.IEPGoal
-IEPGoalID [NVARCHAR](256) NOT NULL
-StudentUSI [INT] NOT NULL
-EducationOrganizationId [BIGINT] NULL
-GoalAchievementPeriodBeginDate [DATE] NULL
-GoalAchievementPeriodEndDate [DATE] NULL
-IDEAEventDescriptorId [INT] NULL
-IDEAEventID [NVARCHAR](1024) NULL
-IEPFinalizedDate [DATE] NOT NULL
-IEPGoalDescriptorId [INT] NOT NULL
-IEPGoalDetails [NVARCHAR](2048) NOT NULL
-IEPServicingEducationOrganizationId [BIGINT] NOT NULL
-StudentIEPAssociationID [NVARCHAR](1024) NOT NULL
-CreateDate [DATETIME] NOT NULL
-LastModifiedDate [DATETIME] NOT NULL
-Id [UNIQUEIDENTIFIER] NOT NULL
-Primary Keys:
-IEPGoalID
-StudentUSI
-</t>
-  </si>
-  <si>
-    <t>IEPServiceDelivery (SEDM)</t>
-  </si>
-  <si>
-    <t>Services delivered to a student as prescribed by their IEP.</t>
-  </si>
-  <si>
-    <t>Contains:
-ExternalServiceProvider (optional collection)
-IDEAEvent (optional)
-IEPServiceDeliveryID (identity)
-IEPServicePrescription (optional)
-ServiceDelivery (identity)
-ServiceDeliveryDate (identity)
-ServiceProvider (optional)
-Staff (optional)
-Student (identity)
-StudentIEPAssociation (required)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sedm.IEPServiceDelivery
-IEPServiceDeliveryID [NVARCHAR](1024) NOT NULL
-ServiceDeliveryDate [DATE] NOT NULL
-ServiceDeliveryDescriptorId [INT] NOT NULL
-StudentUSI [INT] NOT NULL
-EducationOrganizationId [BIGINT] NULL
-IDEAEventDescriptorId [INT] NULL
-IDEAEventID [NVARCHAR](1024) NULL
-IEPFinalizedDate [DATE] NOT NULL
-IEPServicingEducationOrganizationId [BIGINT] NOT NULL
-ServiceDeliveryStaffUSI [INT] NULL
-ServicePrescriptionDate [DATE] NULL
-ServicePrescriptionDescriptorId [INT] NULL
-ServiceProviderDescriptorId [INT] NULL
-StudentIEPAssociationID [NVARCHAR](1024) NOT NULL
-CreateDate [DATETIME] NOT NULL
-LastModifiedDate [DATETIME] NOT NULL
-Id [UNIQUEIDENTIFIER] NOT NULL
-Primary Keys:
-IEPServiceDeliveryID
-ServiceDeliveryDate
-ServiceDeliveryDescriptorId
-StudentUSI
-sedm.IEPServiceDeliveryExternalServiceProvider
-IEPServiceDeliveryID [NVARCHAR](1024) NOT NULL
-ServiceDeliveryDate [DATE] NOT NULL
-ServiceDeliveryDescriptorId [INT] NOT NULL
-StudentUSI [INT] NOT NULL
-ProviderCode [NVARCHAR](1024) NOT NULL
-ProviderFirstName [NVARCHAR](1024) NOT NULL
-ProviderLastSurname [NVARCHAR](1024) NOT NULL
-PrimaryProvider [BIT] NULL
-ProviderMiddleName [NVARCHAR](1024) NULL
-CreateDate [DATETIME] NOT NULL
-Primary Keys:
-IEPServiceDeliveryID
-ServiceDeliveryDate
-ServiceDeliveryDescriptorId
-StudentUSI
-ProviderCode
-ProviderFirstName
-ProviderLastSurname
-</t>
-  </si>
-  <si>
-    <t>IEPServicePrescription (SEDM)</t>
-  </si>
-  <si>
-    <t>The service prescribed to a student as part of their IEP.</t>
-  </si>
-  <si>
-    <t>Contains:
-BeginDate (required)
-DurationMinutes (required)
-DurationPeriod (required)
-EducationOrganization (optional)
-EndDate (optional)
-FrequencyPeriod (required)
-FrequencyValue (required)
-IDEAEvent (optional)
-ServiceLocationType (required)
-ServicePrescription (identity)
-ServicePrescriptionDate (identity)
-Staff (optional)
-Student (identity)
-StudentIEPAssociation (required)
-Used By:
-IEPServiceDelivery.IEPServicePrescription (as optional)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sedm.IEPServicePrescription
-ServicePrescriptionDate [DATE] NOT NULL
-ServicePrescriptionDescriptorId [INT] NOT NULL
-StudentUSI [INT] NOT NULL
-BeginDate [DATE] NOT NULL
-DurationMinutes [DECIMAL](5, 2) NOT NULL
-DurationPeriodDescriptorId [INT] NOT NULL
-EducationOrganizationId [BIGINT] NULL
-EndDate [DATE] NULL
-FrequencyPeriodDescriptorId [INT] NOT NULL
-FrequencyValue [DECIMAL](5, 2) NOT NULL
-IDEAEventDescriptorId [INT] NULL
-IDEAEventID [NVARCHAR](1024) NULL
-IEPFinalizedDate [DATE] NOT NULL
-IEPServicingEducationOrganizationId [BIGINT] NOT NULL
-ServiceLocationTypeDescriptorId [INT] NOT NULL
-ServiceProvidingEducationOrganizationId [BIGINT] NULL
-StaffUSI [INT] NULL
-StudentIEPAssociationID [NVARCHAR](1024) NOT NULL
-CreateDate [DATETIME] NOT NULL
-LastModifiedDate [DATETIME] NOT NULL
-Id [UNIQUEIDENTIFIER] NOT NULL
-Primary Keys:
-ServicePrescriptionDate
-ServicePrescriptionDescriptorId
-StudentUSI
-</t>
-  </si>
-  <si>
-    <t>StudentIEPAccommodation (SEDM)</t>
-  </si>
-  <si>
-    <t>The accommodations prescribed to a student as part of their IEP.</t>
-  </si>
-  <si>
-    <t>Contains:
-Accommodation (required collection)
-EducationOrganization (identity)
-Student (identity)
-StudentIEPAssociation (required)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sedm.StudentIEPAccommodation
-IEPServicingEducationOrganizationId [BIGINT] NOT NULL
-StudentUSI [INT] NOT NULL
-AccommodationDescriptorId [INT] NOT NULL
-CreateDate [DATETIME] NOT NULL
-Primary Keys:
-IEPServicingEducationOrganizationId
-StudentUSI
-AccommodationDescriptorId
-sedm.StudentIEPAccommodation
-IEPServicingEducationOrganizationId [BIGINT] NOT NULL
-StudentUSI [INT] NOT NULL
-IEPFinalizedDate [DATE] NOT NULL
-StudentIEPAssociationID [NVARCHAR](1024) NOT NULL
-CreateDate [DATETIME] NOT NULL
-LastModifiedDate [DATETIME] NOT NULL
-Id [UNIQUEIDENTIFIER] NOT NULL
-Primary Keys:
-IEPServicingEducationOrganizationId
-StudentUSI
-</t>
-  </si>
-  <si>
-    <t>StudentIEPDisability (SEDM)</t>
-  </si>
-  <si>
-    <t>The disabilities prescribed to a student as part of their IEP.</t>
-  </si>
-  <si>
-    <t>Contains:
-Disability (required collection)
-EducationOrganization (identity)
-Student (identity)
-StudentIEPAssociation (required)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sedm.StudentIEPDisability
-IEPServicingEducationOrganizationId [BIGINT] NOT NULL
-StudentUSI [INT] NOT NULL
-DisabilityDescriptorId [INT] NOT NULL
-DisabilityDeterminationSourceTypeDescriptorId [INT] NULL
-DisabilityDiagnosis [NVARCHAR](80) NULL
-OrderOfDisability [INT] NULL
-CreateDate [DATETIME] NOT NULL
-Primary Keys:
-IEPServicingEducationOrganizationId
-StudentUSI
-DisabilityDescriptorId
-sedm.StudentIEPDisability
-IEPServicingEducationOrganizationId [BIGINT] NOT NULL
-StudentUSI [INT] NOT NULL
-IEPFinalizedDate [DATE] NOT NULL
-StudentIEPAssociationID [NVARCHAR](1024) NOT NULL
-CreateDate [DATETIME] NOT NULL
-LastModifiedDate [DATETIME] NOT NULL
-Id [UNIQUEIDENTIFIER] NOT NULL
-Primary Keys:
-IEPServicingEducationOrganizationId
-StudentUSI
-sedm.StudentIEPDisabilityDesignation
-IEPServicingEducationOrganizationId [BIGINT] NOT NULL
-StudentUSI [INT] NOT NULL
-DisabilityDescriptorId [INT] NOT NULL
-DisabilityDesignationDescriptorId [INT] NOT NULL
-CreateDate [DATETIME] NOT NULL
-Primary Keys:
-IEPServicingEducationOrganizationId
-StudentUSI
-DisabilityDescriptorId
-DisabilityDesignationDescriptorId
-</t>
+    <t>IEPGoalID</t>
+  </si>
+  <si>
+    <t>A unique identifier assigned by the provider of IEP services.</t>
+  </si>
+  <si>
+    <t>max length: 256</t>
+  </si>
+  <si>
+    <t>IEPGoalID [NVARCHAR](256)</t>
+  </si>
+  <si>
+    <t>IEPGoalDetails</t>
+  </si>
+  <si>
+    <t>Instructions or other details specific to the student and/or provider for achieving the stated goal.</t>
+  </si>
+  <si>
+    <t>IEPGoalDetails [NVARCHAR](2048)</t>
+  </si>
+  <si>
+    <t>IEPServiceDeliveryID</t>
+  </si>
+  <si>
+    <t>A unique identifier assigned by the provider of IEP services for the delivery record.</t>
+  </si>
+  <si>
+    <t>IEPServiceDeliveryID [NVARCHAR](1024)</t>
+  </si>
+  <si>
+    <t>ProviderCode</t>
+  </si>
+  <si>
+    <t>A code assigned to the external service provider.</t>
+  </si>
+  <si>
+    <t>ProviderCode [NVARCHAR](1024)</t>
+  </si>
+  <si>
+    <t>ProviderFirstName</t>
+  </si>
+  <si>
+    <t>The first name of the external service provider.</t>
+  </si>
+  <si>
+    <t>ProviderFirstName [NVARCHAR](1024)</t>
+  </si>
+  <si>
+    <t>ProviderLastSurname</t>
+  </si>
+  <si>
+    <t>The last name of the external service provider.</t>
+  </si>
+  <si>
+    <t>ProviderLastSurname [NVARCHAR](1024)</t>
+  </si>
+  <si>
+    <t>ProviderMiddleName</t>
+  </si>
+  <si>
+    <t>The middle name of the external service provider.</t>
+  </si>
+  <si>
+    <t>ProviderMiddleName [NVARCHAR](1024)</t>
+  </si>
+  <si>
+    <t>IDEAEventID</t>
+  </si>
+  <si>
+    <t>A unique identifier for the event record as assigned by the provider of IEP services.</t>
+  </si>
+  <si>
+    <t>IDEAEventID [NVARCHAR](1024)</t>
+  </si>
+  <si>
+    <t>EventNarrative</t>
+  </si>
+  <si>
+    <t>Detailed and summary notes recorded during the event.</t>
+  </si>
+  <si>
+    <t>EventNarrative [NVARCHAR](2048)</t>
   </si>
   <si>
     <t>StudentIEPAssociationID</t>
@@ -19241,90 +19427,6 @@
   </si>
   <si>
     <t>StudentIEPAssociationID [NVARCHAR](1024)</t>
-  </si>
-  <si>
-    <t>ProviderCode</t>
-  </si>
-  <si>
-    <t>A code assigned to the external service provider.</t>
-  </si>
-  <si>
-    <t>ProviderCode [NVARCHAR](1024)</t>
-  </si>
-  <si>
-    <t>ProviderFirstName</t>
-  </si>
-  <si>
-    <t>The first name of the external service provider.</t>
-  </si>
-  <si>
-    <t>ProviderFirstName [NVARCHAR](1024)</t>
-  </si>
-  <si>
-    <t>ProviderLastSurname</t>
-  </si>
-  <si>
-    <t>The last name of the external service provider.</t>
-  </si>
-  <si>
-    <t>ProviderLastSurname [NVARCHAR](1024)</t>
-  </si>
-  <si>
-    <t>ProviderMiddleName</t>
-  </si>
-  <si>
-    <t>The middle name of the external service provider.</t>
-  </si>
-  <si>
-    <t>ProviderMiddleName [NVARCHAR](1024)</t>
-  </si>
-  <si>
-    <t>IDEAEventID</t>
-  </si>
-  <si>
-    <t>A unique identifier for the event record as assigned by the provider of IEP services.</t>
-  </si>
-  <si>
-    <t>IDEAEventID [NVARCHAR](1024)</t>
-  </si>
-  <si>
-    <t>EventNarrative</t>
-  </si>
-  <si>
-    <t>Detailed and summary notes recorded during the event.</t>
-  </si>
-  <si>
-    <t>EventNarrative [NVARCHAR](2048)</t>
-  </si>
-  <si>
-    <t>IEPGoalID</t>
-  </si>
-  <si>
-    <t>A unique identifier assigned by the provider of IEP services.</t>
-  </si>
-  <si>
-    <t>max length: 256</t>
-  </si>
-  <si>
-    <t>IEPGoalID [NVARCHAR](256)</t>
-  </si>
-  <si>
-    <t>IEPGoalDetails</t>
-  </si>
-  <si>
-    <t>Instructions or other details specific to the student and/or provider for achieving the stated goal.</t>
-  </si>
-  <si>
-    <t>IEPGoalDetails [NVARCHAR](2048)</t>
-  </si>
-  <si>
-    <t>IEPServiceDeliveryID</t>
-  </si>
-  <si>
-    <t>A unique identifier assigned by the provider of IEP services for the delivery record.</t>
-  </si>
-  <si>
-    <t>IEPServiceDeliveryID [NVARCHAR](1024)</t>
   </si>
 </sst>
 </file>
@@ -33904,370 +34006,370 @@
     </row>
     <row r="878">
       <c r="A878" t="s">
-        <v>310</v>
+        <v>3077</v>
       </c>
       <c r="B878" t="s">
-        <v>311</v>
+        <v>3078</v>
       </c>
       <c r="C878" t="s">
-        <v>183</v>
+        <v>9</v>
       </c>
       <c r="F878" t="s">
-        <v>3077</v>
+        <v>3079</v>
       </c>
       <c r="G878" t="s">
-        <v>313</v>
+        <v>3080</v>
       </c>
     </row>
     <row r="879">
       <c r="A879" t="s">
-        <v>306</v>
+        <v>3081</v>
       </c>
       <c r="B879" t="s">
-        <v>307</v>
+        <v>3082</v>
       </c>
       <c r="C879" t="s">
-        <v>183</v>
+        <v>9</v>
       </c>
       <c r="F879" t="s">
-        <v>3078</v>
+        <v>3083</v>
       </c>
       <c r="G879" t="s">
-        <v>309</v>
+        <v>3084</v>
       </c>
     </row>
     <row r="880">
       <c r="A880" t="s">
-        <v>366</v>
+        <v>3085</v>
       </c>
       <c r="B880" t="s">
-        <v>3079</v>
+        <v>3086</v>
       </c>
       <c r="C880" t="s">
-        <v>183</v>
+        <v>9</v>
       </c>
       <c r="F880" t="s">
-        <v>3080</v>
+        <v>3087</v>
       </c>
       <c r="G880" t="s">
-        <v>369</v>
+        <v>3088</v>
       </c>
     </row>
     <row r="881">
       <c r="A881" t="s">
-        <v>3081</v>
+        <v>3089</v>
       </c>
       <c r="B881" t="s">
-        <v>3082</v>
+        <v>3090</v>
       </c>
       <c r="C881" t="s">
-        <v>439</v>
+        <v>9</v>
       </c>
       <c r="F881" t="s">
-        <v>3083</v>
+        <v>3091</v>
+      </c>
+      <c r="G881" t="s">
+        <v>3092</v>
       </c>
     </row>
     <row r="882">
       <c r="A882" t="s">
-        <v>3084</v>
+        <v>366</v>
       </c>
       <c r="B882" t="s">
-        <v>3085</v>
+        <v>3093</v>
       </c>
       <c r="C882" t="s">
-        <v>682</v>
+        <v>183</v>
       </c>
       <c r="F882" t="s">
-        <v>3086</v>
+        <v>3094</v>
       </c>
       <c r="G882" t="s">
-        <v>3087</v>
+        <v>369</v>
       </c>
     </row>
     <row r="883">
       <c r="A883" t="s">
-        <v>841</v>
+        <v>310</v>
       </c>
       <c r="B883" t="s">
-        <v>3088</v>
+        <v>311</v>
       </c>
       <c r="C883" t="s">
-        <v>682</v>
+        <v>183</v>
       </c>
       <c r="F883" t="s">
-        <v>3089</v>
+        <v>3095</v>
       </c>
       <c r="G883" t="s">
-        <v>844</v>
+        <v>313</v>
       </c>
     </row>
     <row r="884">
       <c r="A884" t="s">
-        <v>845</v>
+        <v>306</v>
       </c>
       <c r="B884" t="s">
-        <v>3090</v>
+        <v>307</v>
       </c>
       <c r="C884" t="s">
-        <v>682</v>
+        <v>183</v>
       </c>
       <c r="F884" t="s">
-        <v>3091</v>
+        <v>3096</v>
       </c>
       <c r="G884" t="s">
-        <v>848</v>
+        <v>309</v>
       </c>
     </row>
     <row r="885">
       <c r="A885" t="s">
-        <v>3092</v>
+        <v>3097</v>
       </c>
       <c r="B885" t="s">
-        <v>3093</v>
+        <v>3098</v>
       </c>
       <c r="C885" t="s">
-        <v>682</v>
+        <v>439</v>
       </c>
       <c r="F885" t="s">
-        <v>3094</v>
-      </c>
-      <c r="G885" t="s">
-        <v>3095</v>
+        <v>3099</v>
       </c>
     </row>
     <row r="886">
       <c r="A886" t="s">
-        <v>3096</v>
+        <v>3100</v>
       </c>
       <c r="B886" t="s">
-        <v>3097</v>
+        <v>3101</v>
       </c>
       <c r="C886" t="s">
         <v>682</v>
       </c>
       <c r="F886" t="s">
-        <v>3098</v>
+        <v>3102</v>
       </c>
       <c r="G886" t="s">
-        <v>3099</v>
+        <v>3103</v>
       </c>
     </row>
     <row r="887">
       <c r="A887" t="s">
-        <v>3100</v>
+        <v>3104</v>
       </c>
       <c r="B887" t="s">
-        <v>3101</v>
+        <v>3105</v>
       </c>
       <c r="C887" t="s">
         <v>682</v>
       </c>
       <c r="F887" t="s">
-        <v>3102</v>
+        <v>3106</v>
       </c>
       <c r="G887" t="s">
-        <v>3103</v>
+        <v>3107</v>
       </c>
     </row>
     <row r="888">
       <c r="A888" t="s">
-        <v>3104</v>
+        <v>3108</v>
       </c>
       <c r="B888" t="s">
-        <v>3105</v>
+        <v>3109</v>
       </c>
       <c r="C888" t="s">
         <v>682</v>
       </c>
       <c r="F888" t="s">
-        <v>3106</v>
+        <v>3110</v>
       </c>
       <c r="G888" t="s">
-        <v>3107</v>
+        <v>3111</v>
       </c>
     </row>
     <row r="889">
       <c r="A889" t="s">
-        <v>3108</v>
+        <v>3112</v>
       </c>
       <c r="B889" t="s">
-        <v>3109</v>
+        <v>3113</v>
       </c>
       <c r="C889" t="s">
         <v>682</v>
       </c>
       <c r="F889" t="s">
-        <v>3110</v>
+        <v>3114</v>
       </c>
       <c r="G889" t="s">
-        <v>3111</v>
+        <v>3115</v>
       </c>
     </row>
     <row r="890">
       <c r="A890" t="s">
-        <v>3112</v>
+        <v>3116</v>
       </c>
       <c r="B890" t="s">
-        <v>3113</v>
+        <v>3117</v>
       </c>
       <c r="C890" t="s">
         <v>682</v>
       </c>
       <c r="F890" t="s">
-        <v>3114</v>
+        <v>3118</v>
       </c>
       <c r="G890" t="s">
-        <v>3115</v>
+        <v>684</v>
       </c>
     </row>
     <row r="891">
       <c r="A891" t="s">
-        <v>3116</v>
+        <v>3119</v>
       </c>
       <c r="B891" t="s">
-        <v>3117</v>
+        <v>3120</v>
       </c>
       <c r="C891" t="s">
         <v>682</v>
       </c>
       <c r="F891" t="s">
-        <v>3118</v>
+        <v>3121</v>
       </c>
       <c r="G891" t="s">
-        <v>3119</v>
+        <v>688</v>
       </c>
     </row>
     <row r="892">
       <c r="A892" t="s">
-        <v>3120</v>
+        <v>3122</v>
       </c>
       <c r="B892" t="s">
-        <v>3121</v>
+        <v>3123</v>
       </c>
       <c r="C892" t="s">
         <v>682</v>
       </c>
       <c r="F892" t="s">
-        <v>3122</v>
+        <v>3124</v>
       </c>
       <c r="G892" t="s">
-        <v>684</v>
+        <v>3125</v>
       </c>
     </row>
     <row r="893">
       <c r="A893" t="s">
-        <v>3123</v>
+        <v>3126</v>
       </c>
       <c r="B893" t="s">
-        <v>3124</v>
+        <v>3127</v>
       </c>
       <c r="C893" t="s">
         <v>682</v>
       </c>
       <c r="F893" t="s">
-        <v>3125</v>
+        <v>3128</v>
       </c>
       <c r="G893" t="s">
-        <v>688</v>
+        <v>3129</v>
       </c>
     </row>
     <row r="894">
       <c r="A894" t="s">
-        <v>3126</v>
+        <v>3130</v>
       </c>
       <c r="B894" t="s">
-        <v>3127</v>
+        <v>3131</v>
       </c>
       <c r="C894" t="s">
-        <v>1139</v>
-      </c>
-      <c r="D894" t="s">
-        <v>1144</v>
+        <v>682</v>
+      </c>
+      <c r="F894" t="s">
+        <v>3132</v>
       </c>
       <c r="G894" t="s">
-        <v>3128</v>
+        <v>3133</v>
       </c>
     </row>
     <row r="895">
       <c r="A895" t="s">
-        <v>3129</v>
+        <v>841</v>
       </c>
       <c r="B895" t="s">
-        <v>3130</v>
+        <v>3134</v>
       </c>
       <c r="C895" t="s">
-        <v>1139</v>
-      </c>
-      <c r="D895" t="s">
-        <v>1144</v>
+        <v>682</v>
+      </c>
+      <c r="F895" t="s">
+        <v>3135</v>
       </c>
       <c r="G895" t="s">
-        <v>3131</v>
+        <v>844</v>
       </c>
     </row>
     <row r="896">
       <c r="A896" t="s">
-        <v>3132</v>
+        <v>845</v>
       </c>
       <c r="B896" t="s">
-        <v>3133</v>
+        <v>3136</v>
       </c>
       <c r="C896" t="s">
-        <v>1208</v>
+        <v>682</v>
       </c>
       <c r="F896" t="s">
-        <v>3134</v>
+        <v>3137</v>
       </c>
       <c r="G896" t="s">
-        <v>3135</v>
+        <v>848</v>
       </c>
     </row>
     <row r="897">
       <c r="A897" t="s">
-        <v>3136</v>
+        <v>3138</v>
       </c>
       <c r="B897" t="s">
-        <v>3137</v>
+        <v>3139</v>
       </c>
       <c r="C897" t="s">
-        <v>1208</v>
+        <v>682</v>
       </c>
       <c r="F897" t="s">
-        <v>3138</v>
+        <v>3140</v>
       </c>
       <c r="G897" t="s">
-        <v>3139</v>
+        <v>3141</v>
       </c>
     </row>
     <row r="898">
       <c r="A898" t="s">
-        <v>3140</v>
+        <v>3142</v>
       </c>
       <c r="B898" t="s">
-        <v>3141</v>
+        <v>3143</v>
       </c>
       <c r="C898" t="s">
-        <v>1208</v>
-      </c>
-      <c r="F898" t="s">
-        <v>3142</v>
+        <v>1139</v>
+      </c>
+      <c r="D898" t="s">
+        <v>1144</v>
       </c>
       <c r="G898" t="s">
-        <v>3143</v>
+        <v>3144</v>
       </c>
     </row>
     <row r="899">
       <c r="A899" t="s">
-        <v>3144</v>
+        <v>3145</v>
       </c>
       <c r="B899" t="s">
-        <v>3145</v>
+        <v>3146</v>
       </c>
       <c r="C899" t="s">
-        <v>1208</v>
-      </c>
-      <c r="F899" t="s">
-        <v>3146</v>
+        <v>1139</v>
+      </c>
+      <c r="D899" t="s">
+        <v>1144</v>
       </c>
       <c r="G899" t="s">
         <v>3147</v>
@@ -34334,73 +34436,73 @@
       <c r="C903" t="s">
         <v>1208</v>
       </c>
+      <c r="F903" t="s">
+        <v>3162</v>
+      </c>
       <c r="G903" t="s">
-        <v>3162</v>
+        <v>3163</v>
       </c>
     </row>
     <row r="904">
       <c r="A904" t="s">
-        <v>3163</v>
+        <v>3164</v>
       </c>
       <c r="B904" t="s">
-        <v>3164</v>
+        <v>3165</v>
       </c>
       <c r="C904" t="s">
         <v>1208</v>
       </c>
       <c r="F904" t="s">
-        <v>3165</v>
+        <v>3166</v>
       </c>
       <c r="G904" t="s">
-        <v>3166</v>
+        <v>3167</v>
       </c>
     </row>
     <row r="905">
       <c r="A905" t="s">
-        <v>3167</v>
+        <v>3168</v>
       </c>
       <c r="B905" t="s">
-        <v>3168</v>
+        <v>3169</v>
       </c>
       <c r="C905" t="s">
         <v>1208</v>
       </c>
       <c r="F905" t="s">
-        <v>3169</v>
+        <v>3170</v>
       </c>
       <c r="G905" t="s">
-        <v>3170</v>
+        <v>3171</v>
       </c>
     </row>
     <row r="906">
       <c r="A906" t="s">
-        <v>3171</v>
+        <v>3172</v>
       </c>
       <c r="B906" t="s">
-        <v>3172</v>
+        <v>3173</v>
       </c>
       <c r="C906" t="s">
         <v>1208</v>
       </c>
       <c r="F906" t="s">
-        <v>3173</v>
+        <v>3174</v>
       </c>
       <c r="G906" t="s">
-        <v>3174</v>
+        <v>3175</v>
       </c>
     </row>
     <row r="907">
       <c r="A907" t="s">
-        <v>3175</v>
+        <v>3176</v>
       </c>
       <c r="B907" t="s">
-        <v>3176</v>
+        <v>3177</v>
       </c>
       <c r="C907" t="s">
         <v>1208</v>
-      </c>
-      <c r="F907" t="s">
-        <v>3177</v>
       </c>
       <c r="G907" t="s">
         <v>3178</v>
@@ -34416,152 +34518,152 @@
       <c r="C908" t="s">
         <v>1208</v>
       </c>
+      <c r="F908" t="s">
+        <v>3181</v>
+      </c>
       <c r="G908" t="s">
-        <v>3181</v>
+        <v>3182</v>
       </c>
     </row>
     <row r="909">
       <c r="A909" t="s">
-        <v>3148</v>
+        <v>3183</v>
       </c>
       <c r="B909" t="s">
-        <v>3182</v>
+        <v>3184</v>
       </c>
       <c r="C909" t="s">
-        <v>2036</v>
+        <v>1208</v>
       </c>
       <c r="F909" t="s">
-        <v>3183</v>
+        <v>3185</v>
       </c>
       <c r="G909" t="s">
-        <v>3184</v>
+        <v>3186</v>
       </c>
     </row>
     <row r="910">
       <c r="A910" t="s">
-        <v>3152</v>
+        <v>3187</v>
       </c>
       <c r="B910" t="s">
-        <v>3185</v>
+        <v>3188</v>
       </c>
       <c r="C910" t="s">
-        <v>2036</v>
+        <v>1208</v>
       </c>
       <c r="F910" t="s">
-        <v>3186</v>
+        <v>3189</v>
       </c>
       <c r="G910" t="s">
-        <v>3187</v>
+        <v>3190</v>
       </c>
     </row>
     <row r="911">
       <c r="A911" t="s">
-        <v>3188</v>
+        <v>3191</v>
       </c>
       <c r="B911" t="s">
-        <v>3189</v>
+        <v>3192</v>
       </c>
       <c r="C911" t="s">
-        <v>2036</v>
+        <v>1208</v>
       </c>
       <c r="F911" t="s">
-        <v>3190</v>
+        <v>3193</v>
       </c>
       <c r="G911" t="s">
-        <v>3191</v>
+        <v>3194</v>
       </c>
     </row>
     <row r="912">
       <c r="A912" t="s">
-        <v>3192</v>
+        <v>3195</v>
       </c>
       <c r="B912" t="s">
-        <v>3193</v>
+        <v>3196</v>
       </c>
       <c r="C912" t="s">
-        <v>2036</v>
-      </c>
-      <c r="F912" t="s">
-        <v>3194</v>
+        <v>1208</v>
       </c>
       <c r="G912" t="s">
-        <v>3195</v>
+        <v>3197</v>
       </c>
     </row>
     <row r="913">
       <c r="A913" t="s">
-        <v>3196</v>
+        <v>3164</v>
       </c>
       <c r="B913" t="s">
-        <v>3197</v>
+        <v>3198</v>
       </c>
       <c r="C913" t="s">
         <v>2036</v>
       </c>
       <c r="F913" t="s">
-        <v>3198</v>
+        <v>3199</v>
       </c>
       <c r="G913" t="s">
-        <v>3199</v>
+        <v>3200</v>
       </c>
     </row>
     <row r="914">
       <c r="A914" t="s">
-        <v>3200</v>
+        <v>3201</v>
       </c>
       <c r="B914" t="s">
-        <v>3201</v>
+        <v>3202</v>
       </c>
       <c r="C914" t="s">
         <v>2036</v>
       </c>
       <c r="F914" t="s">
-        <v>3202</v>
+        <v>3203</v>
       </c>
       <c r="G914" t="s">
-        <v>3203</v>
+        <v>3204</v>
       </c>
     </row>
     <row r="915">
       <c r="A915" t="s">
-        <v>3204</v>
+        <v>3205</v>
       </c>
       <c r="B915" t="s">
-        <v>3205</v>
+        <v>3206</v>
       </c>
       <c r="C915" t="s">
         <v>2606</v>
       </c>
       <c r="D915" t="s">
-        <v>2615</v>
+        <v>3207</v>
       </c>
       <c r="G915" t="s">
-        <v>3206</v>
+        <v>3208</v>
       </c>
     </row>
     <row r="916">
       <c r="A916" t="s">
-        <v>3207</v>
+        <v>3209</v>
       </c>
       <c r="B916" t="s">
-        <v>3208</v>
+        <v>3210</v>
       </c>
       <c r="C916" t="s">
         <v>2606</v>
       </c>
       <c r="D916" t="s">
-        <v>2615</v>
+        <v>3012</v>
       </c>
       <c r="G916" t="s">
-        <v>3209</v>
+        <v>3211</v>
       </c>
     </row>
     <row r="917">
       <c r="A917" t="s">
-        <v>3210</v>
+        <v>3212</v>
       </c>
       <c r="B917" t="s">
-        <v>3211</v>
+        <v>3213</v>
       </c>
       <c r="C917" t="s">
         <v>2606</v>
@@ -34570,15 +34672,15 @@
         <v>2615</v>
       </c>
       <c r="G917" t="s">
-        <v>3212</v>
+        <v>3214</v>
       </c>
     </row>
     <row r="918">
       <c r="A918" t="s">
-        <v>3213</v>
+        <v>3215</v>
       </c>
       <c r="B918" t="s">
-        <v>3214</v>
+        <v>3216</v>
       </c>
       <c r="C918" t="s">
         <v>2606</v>
@@ -34587,15 +34689,15 @@
         <v>2615</v>
       </c>
       <c r="G918" t="s">
-        <v>3215</v>
+        <v>3217</v>
       </c>
     </row>
     <row r="919">
       <c r="A919" t="s">
-        <v>3216</v>
+        <v>3218</v>
       </c>
       <c r="B919" t="s">
-        <v>3217</v>
+        <v>3219</v>
       </c>
       <c r="C919" t="s">
         <v>2606</v>
@@ -34604,15 +34706,15 @@
         <v>2615</v>
       </c>
       <c r="G919" t="s">
-        <v>3218</v>
+        <v>3220</v>
       </c>
     </row>
     <row r="920">
       <c r="A920" t="s">
-        <v>3219</v>
+        <v>3221</v>
       </c>
       <c r="B920" t="s">
-        <v>3220</v>
+        <v>3222</v>
       </c>
       <c r="C920" t="s">
         <v>2606</v>
@@ -34621,49 +34723,49 @@
         <v>2615</v>
       </c>
       <c r="G920" t="s">
-        <v>3221</v>
+        <v>3223</v>
       </c>
     </row>
     <row r="921">
       <c r="A921" t="s">
-        <v>3222</v>
+        <v>3224</v>
       </c>
       <c r="B921" t="s">
-        <v>3223</v>
+        <v>3225</v>
       </c>
       <c r="C921" t="s">
         <v>2606</v>
       </c>
       <c r="D921" t="s">
-        <v>3012</v>
+        <v>2615</v>
       </c>
       <c r="G921" t="s">
-        <v>3224</v>
+        <v>3226</v>
       </c>
     </row>
     <row r="922">
       <c r="A922" t="s">
-        <v>3225</v>
+        <v>3227</v>
       </c>
       <c r="B922" t="s">
-        <v>3226</v>
+        <v>3228</v>
       </c>
       <c r="C922" t="s">
         <v>2606</v>
       </c>
       <c r="D922" t="s">
-        <v>3227</v>
+        <v>2615</v>
       </c>
       <c r="G922" t="s">
-        <v>3228</v>
+        <v>3229</v>
       </c>
     </row>
     <row r="923">
       <c r="A923" t="s">
-        <v>3229</v>
+        <v>3230</v>
       </c>
       <c r="B923" t="s">
-        <v>3230</v>
+        <v>3231</v>
       </c>
       <c r="C923" t="s">
         <v>2606</v>
@@ -34672,15 +34774,15 @@
         <v>3012</v>
       </c>
       <c r="G923" t="s">
-        <v>3231</v>
+        <v>3232</v>
       </c>
     </row>
     <row r="924">
       <c r="A924" t="s">
-        <v>3232</v>
+        <v>3233</v>
       </c>
       <c r="B924" t="s">
-        <v>3233</v>
+        <v>3234</v>
       </c>
       <c r="C924" t="s">
         <v>2606</v>
@@ -34689,7 +34791,7 @@
         <v>2615</v>
       </c>
       <c r="G924" t="s">
-        <v>3234</v>
+        <v>3235</v>
       </c>
     </row>
   </sheetData>

</xml_diff>